<commit_message>
fix | Database Export | flipped relationship direction
</commit_message>
<xml_diff>
--- a/storage/app/templates/burial-assistances-template.xlsx
+++ b/storage/app/templates/burial-assistances-template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\burial\storage\app\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E2F4045-5CE8-41DE-AA20-32EC2553CA9F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="40" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2128B93-D8CA-45CA-AA8B-3784688F220E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="40" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9648" xr2:uid="{AD9B507F-99D9-4301-BBEB-177307A70AB4}"/>
   </bookViews>
@@ -51,9 +51,6 @@
     <t>EXT</t>
   </si>
   <si>
-    <t>RELATIONSHIP OF DECEASED TO THE CLAIMANT</t>
-  </si>
-  <si>
     <t>DATE OF BIRTH</t>
   </si>
   <si>
@@ -175,6 +172,9 @@
   </si>
   <si>
     <t xml:space="preserve">OBR </t>
+  </si>
+  <si>
+    <t>RELATIONSHIP OF CLAIMANT TO THE DECEASED</t>
   </si>
 </sst>
 </file>
@@ -551,25 +551,58 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -591,39 +624,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
   </cellXfs>
@@ -987,149 +987,149 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:65" s="7" customFormat="1" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="D1" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="E1" s="30" t="s">
         <v>40</v>
       </c>
-      <c r="E1" s="19" t="s">
+      <c r="F1" s="31"/>
+      <c r="G1" s="31"/>
+      <c r="H1" s="32"/>
+      <c r="I1" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="21"/>
-      <c r="I1" s="15" t="s">
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
+      <c r="L1" s="18"/>
+      <c r="M1" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="N1" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="O1" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="P1" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="Q1" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="R1" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="S1" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="T1" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="U1" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="V1" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="W1" s="23" t="s">
+        <v>16</v>
+      </c>
+      <c r="X1" s="24"/>
+      <c r="Y1" s="25"/>
+      <c r="Z1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA1" s="23" t="s">
+        <v>18</v>
+      </c>
+      <c r="AB1" s="24"/>
+      <c r="AC1" s="25"/>
+      <c r="AD1" s="23" t="s">
+        <v>16</v>
+      </c>
+      <c r="AE1" s="24"/>
+      <c r="AF1" s="24"/>
+      <c r="AG1" s="24"/>
+      <c r="AH1" s="25"/>
+      <c r="AI1" s="23" t="s">
+        <v>19</v>
+      </c>
+      <c r="AJ1" s="25"/>
+      <c r="AK1" s="23" t="s">
+        <v>20</v>
+      </c>
+      <c r="AL1" s="25"/>
+      <c r="AM1" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="AN1" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="J1" s="15"/>
-      <c r="K1" s="15"/>
-      <c r="L1" s="16"/>
-      <c r="M1" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="N1" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="O1" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="P1" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="Q1" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="R1" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="S1" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="T1" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="U1" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="V1" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="W1" s="24" t="s">
-        <v>17</v>
-      </c>
-      <c r="X1" s="25"/>
-      <c r="Y1" s="26"/>
-      <c r="Z1" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="AA1" s="24" t="s">
-        <v>19</v>
-      </c>
-      <c r="AB1" s="25"/>
-      <c r="AC1" s="26"/>
-      <c r="AD1" s="24" t="s">
-        <v>17</v>
-      </c>
-      <c r="AE1" s="25"/>
-      <c r="AF1" s="25"/>
-      <c r="AG1" s="25"/>
-      <c r="AH1" s="26"/>
-      <c r="AI1" s="24" t="s">
-        <v>20</v>
-      </c>
-      <c r="AJ1" s="26"/>
-      <c r="AK1" s="24" t="s">
+      <c r="AO1" s="17"/>
+      <c r="AP1" s="18"/>
+      <c r="AQ1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="AL1" s="26"/>
-      <c r="AM1" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="AN1" s="13" t="s">
+      <c r="AR1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="AS1" s="23" t="s">
+        <v>23</v>
+      </c>
+      <c r="AT1" s="25"/>
+      <c r="AU1" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="AV1" s="23" t="s">
+        <v>25</v>
+      </c>
+      <c r="AW1" s="24"/>
+      <c r="AX1" s="24"/>
+      <c r="AY1" s="24"/>
+      <c r="AZ1" s="24"/>
+      <c r="BA1" s="24"/>
+      <c r="BB1" s="24"/>
+      <c r="BC1" s="24"/>
+      <c r="BD1" s="24"/>
+      <c r="BE1" s="24"/>
+      <c r="BF1" s="24"/>
+      <c r="BG1" s="24"/>
+      <c r="BH1" s="24"/>
+      <c r="BI1" s="24"/>
+      <c r="BJ1" s="25"/>
+      <c r="BK1" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="BL1" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="BM1" s="10" t="s">
         <v>43</v>
-      </c>
-      <c r="AO1" s="15"/>
-      <c r="AP1" s="16"/>
-      <c r="AQ1" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="AR1" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="AS1" s="24" t="s">
-        <v>24</v>
-      </c>
-      <c r="AT1" s="26"/>
-      <c r="AU1" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="AV1" s="24" t="s">
-        <v>26</v>
-      </c>
-      <c r="AW1" s="25"/>
-      <c r="AX1" s="25"/>
-      <c r="AY1" s="25"/>
-      <c r="AZ1" s="25"/>
-      <c r="BA1" s="25"/>
-      <c r="BB1" s="25"/>
-      <c r="BC1" s="25"/>
-      <c r="BD1" s="25"/>
-      <c r="BE1" s="25"/>
-      <c r="BF1" s="25"/>
-      <c r="BG1" s="25"/>
-      <c r="BH1" s="25"/>
-      <c r="BI1" s="25"/>
-      <c r="BJ1" s="26"/>
-      <c r="BK1" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="BL1" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="BM1" s="27" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:65" s="7" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
-      <c r="H2" s="23"/>
-      <c r="I2" s="17"/>
-      <c r="J2" s="17"/>
-      <c r="K2" s="17"/>
-      <c r="L2" s="18"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="28"/>
+      <c r="G2" s="28"/>
+      <c r="H2" s="34"/>
+      <c r="I2" s="28"/>
+      <c r="J2" s="28"/>
+      <c r="K2" s="28"/>
+      <c r="L2" s="29"/>
       <c r="M2" s="11"/>
       <c r="N2" s="11"/>
       <c r="O2" s="11"/>
@@ -1140,111 +1140,111 @@
       <c r="T2" s="11"/>
       <c r="U2" s="11"/>
       <c r="V2" s="11"/>
-      <c r="W2" s="27" t="s">
+      <c r="W2" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="X2" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="X2" s="27" t="s">
+      <c r="Y2" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="Y2" s="27" t="s">
+      <c r="Z2" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="AA2" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="Z2" s="27" t="s">
-        <v>18</v>
-      </c>
-      <c r="AA2" s="27" t="s">
+      <c r="AB2" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="AC2" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="AD2" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="AE2" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="AF2" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="AB2" s="27" t="s">
+      <c r="AG2" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="AH2" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="AC2" s="27" t="s">
-        <v>30</v>
-      </c>
-      <c r="AD2" s="27" t="s">
+      <c r="AI2" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="AJ2" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="AE2" s="27" t="s">
-        <v>30</v>
-      </c>
-      <c r="AF2" s="27" t="s">
-        <v>33</v>
-      </c>
-      <c r="AG2" s="27" t="s">
+      <c r="AK2" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="AL2" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="AH2" s="27" t="s">
-        <v>30</v>
-      </c>
-      <c r="AI2" s="27" t="s">
-        <v>29</v>
-      </c>
-      <c r="AJ2" s="27" t="s">
-        <v>30</v>
-      </c>
-      <c r="AK2" s="27" t="s">
-        <v>29</v>
-      </c>
-      <c r="AL2" s="27" t="s">
-        <v>30</v>
-      </c>
-      <c r="AM2" s="14"/>
-      <c r="AN2" s="33" t="s">
+      <c r="AM2" s="26"/>
+      <c r="AN2" s="19" t="s">
+        <v>46</v>
+      </c>
+      <c r="AO2" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="AO2" s="34" t="s">
-        <v>48</v>
-      </c>
-      <c r="AP2" s="30"/>
-      <c r="AQ2" s="27" t="s">
+      <c r="AP2" s="21"/>
+      <c r="AQ2" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="AR2" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="AS2" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="AR2" s="27" t="s">
-        <v>35</v>
-      </c>
-      <c r="AS2" s="31" t="s">
+      <c r="AT2" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="AT2" s="31" t="s">
+      <c r="AU2" s="11"/>
+      <c r="AV2" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="AW2" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="AX2" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="AY2" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="AZ2" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="AU2" s="11"/>
-      <c r="AV2" s="27" t="s">
-        <v>3</v>
-      </c>
-      <c r="AW2" s="27" t="s">
-        <v>4</v>
-      </c>
-      <c r="AX2" s="27" t="s">
-        <v>5</v>
-      </c>
-      <c r="AY2" s="27" t="s">
-        <v>6</v>
-      </c>
-      <c r="AZ2" s="27" t="s">
+      <c r="BA2" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="BB2" s="21"/>
+      <c r="BC2" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="BD2" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="BE2" s="21"/>
+      <c r="BF2" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="BG2" s="21"/>
+      <c r="BH2" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="BI2" s="21"/>
+      <c r="BJ2" s="10" t="s">
         <v>38</v>
-      </c>
-      <c r="BA2" s="29" t="s">
-        <v>17</v>
-      </c>
-      <c r="BB2" s="30"/>
-      <c r="BC2" s="27" t="s">
-        <v>33</v>
-      </c>
-      <c r="BD2" s="29" t="s">
-        <v>17</v>
-      </c>
-      <c r="BE2" s="30"/>
-      <c r="BF2" s="29" t="s">
-        <v>20</v>
-      </c>
-      <c r="BG2" s="30"/>
-      <c r="BH2" s="29" t="s">
-        <v>21</v>
-      </c>
-      <c r="BI2" s="30"/>
-      <c r="BJ2" s="27" t="s">
-        <v>39</v>
       </c>
       <c r="BK2" s="11"/>
       <c r="BL2" s="11"/>
@@ -1305,18 +1305,18 @@
       <c r="AJ3" s="12"/>
       <c r="AK3" s="12"/>
       <c r="AL3" s="12"/>
-      <c r="AM3" s="28"/>
-      <c r="AN3" s="33"/>
+      <c r="AM3" s="27"/>
+      <c r="AN3" s="19"/>
       <c r="AO3" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="AP3" s="4" t="s">
         <v>34</v>
-      </c>
-      <c r="AP3" s="4" t="s">
-        <v>35</v>
       </c>
       <c r="AQ3" s="12"/>
       <c r="AR3" s="12"/>
-      <c r="AS3" s="32"/>
-      <c r="AT3" s="32"/>
+      <c r="AS3" s="14"/>
+      <c r="AT3" s="14"/>
       <c r="AU3" s="12"/>
       <c r="AV3" s="12"/>
       <c r="AW3" s="12"/>
@@ -1324,29 +1324,29 @@
       <c r="AY3" s="12"/>
       <c r="AZ3" s="12"/>
       <c r="BA3" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="BB3" s="1" t="s">
         <v>29</v>
-      </c>
-      <c r="BB3" s="1" t="s">
-        <v>30</v>
       </c>
       <c r="BC3" s="12"/>
       <c r="BD3" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="BE3" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="BE3" s="1" t="s">
-        <v>30</v>
-      </c>
       <c r="BF3" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="BG3" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="BG3" s="1" t="s">
-        <v>30</v>
-      </c>
       <c r="BH3" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="BI3" s="1" t="s">
         <v>29</v>
-      </c>
-      <c r="BI3" s="1" t="s">
-        <v>30</v>
       </c>
       <c r="BJ3" s="12"/>
       <c r="BK3" s="12"/>
@@ -1690,6 +1690,52 @@
     </row>
   </sheetData>
   <mergeCells count="62">
+    <mergeCell ref="A1:A3"/>
+    <mergeCell ref="B1:B3"/>
+    <mergeCell ref="C1:C3"/>
+    <mergeCell ref="S1:S3"/>
+    <mergeCell ref="Q1:Q3"/>
+    <mergeCell ref="R1:R3"/>
+    <mergeCell ref="D1:D3"/>
+    <mergeCell ref="M1:M3"/>
+    <mergeCell ref="N1:N3"/>
+    <mergeCell ref="O1:O3"/>
+    <mergeCell ref="P1:P3"/>
+    <mergeCell ref="I1:L2"/>
+    <mergeCell ref="E1:H2"/>
+    <mergeCell ref="U1:U3"/>
+    <mergeCell ref="V1:V3"/>
+    <mergeCell ref="W1:Y1"/>
+    <mergeCell ref="AA1:AC1"/>
+    <mergeCell ref="AD1:AH1"/>
+    <mergeCell ref="AD2:AD3"/>
+    <mergeCell ref="AE2:AE3"/>
+    <mergeCell ref="AF2:AF3"/>
+    <mergeCell ref="AG2:AG3"/>
+    <mergeCell ref="AH2:AH3"/>
+    <mergeCell ref="BL1:BL3"/>
+    <mergeCell ref="W2:W3"/>
+    <mergeCell ref="X2:X3"/>
+    <mergeCell ref="Y2:Y3"/>
+    <mergeCell ref="Z2:Z3"/>
+    <mergeCell ref="AA2:AA3"/>
+    <mergeCell ref="AB2:AB3"/>
+    <mergeCell ref="AC2:AC3"/>
+    <mergeCell ref="AI1:AJ1"/>
+    <mergeCell ref="AK1:AL1"/>
+    <mergeCell ref="AM1:AM3"/>
+    <mergeCell ref="AS1:AT1"/>
+    <mergeCell ref="AU1:AU3"/>
+    <mergeCell ref="BC2:BC3"/>
+    <mergeCell ref="BD2:BE2"/>
+    <mergeCell ref="BF2:BG2"/>
+    <mergeCell ref="AV1:BJ1"/>
+    <mergeCell ref="BK1:BK3"/>
+    <mergeCell ref="AW2:AW3"/>
+    <mergeCell ref="AX2:AX3"/>
+    <mergeCell ref="AY2:AY3"/>
+    <mergeCell ref="AZ2:AZ3"/>
+    <mergeCell ref="BA2:BB2"/>
     <mergeCell ref="BM1:BM3"/>
     <mergeCell ref="AQ2:AQ3"/>
     <mergeCell ref="AR2:AR3"/>
@@ -1706,52 +1752,6 @@
     <mergeCell ref="BJ2:BJ3"/>
     <mergeCell ref="AT2:AT3"/>
     <mergeCell ref="AV2:AV3"/>
-    <mergeCell ref="AV1:BJ1"/>
-    <mergeCell ref="BK1:BK3"/>
-    <mergeCell ref="AW2:AW3"/>
-    <mergeCell ref="AX2:AX3"/>
-    <mergeCell ref="AY2:AY3"/>
-    <mergeCell ref="AZ2:AZ3"/>
-    <mergeCell ref="BA2:BB2"/>
-    <mergeCell ref="BL1:BL3"/>
-    <mergeCell ref="W2:W3"/>
-    <mergeCell ref="X2:X3"/>
-    <mergeCell ref="Y2:Y3"/>
-    <mergeCell ref="Z2:Z3"/>
-    <mergeCell ref="AA2:AA3"/>
-    <mergeCell ref="AB2:AB3"/>
-    <mergeCell ref="AC2:AC3"/>
-    <mergeCell ref="AI1:AJ1"/>
-    <mergeCell ref="AK1:AL1"/>
-    <mergeCell ref="AM1:AM3"/>
-    <mergeCell ref="AS1:AT1"/>
-    <mergeCell ref="AU1:AU3"/>
-    <mergeCell ref="BC2:BC3"/>
-    <mergeCell ref="BD2:BE2"/>
-    <mergeCell ref="BF2:BG2"/>
-    <mergeCell ref="U1:U3"/>
-    <mergeCell ref="V1:V3"/>
-    <mergeCell ref="W1:Y1"/>
-    <mergeCell ref="AA1:AC1"/>
-    <mergeCell ref="AD1:AH1"/>
-    <mergeCell ref="AD2:AD3"/>
-    <mergeCell ref="AE2:AE3"/>
-    <mergeCell ref="AF2:AF3"/>
-    <mergeCell ref="AG2:AG3"/>
-    <mergeCell ref="AH2:AH3"/>
-    <mergeCell ref="A1:A3"/>
-    <mergeCell ref="B1:B3"/>
-    <mergeCell ref="C1:C3"/>
-    <mergeCell ref="S1:S3"/>
-    <mergeCell ref="Q1:Q3"/>
-    <mergeCell ref="R1:R3"/>
-    <mergeCell ref="D1:D3"/>
-    <mergeCell ref="M1:M3"/>
-    <mergeCell ref="N1:N3"/>
-    <mergeCell ref="O1:O3"/>
-    <mergeCell ref="P1:P3"/>
-    <mergeCell ref="I1:L2"/>
-    <mergeCell ref="E1:H2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="203" r:id="rId1"/>

</xml_diff>